<commit_message>
feat(recuriter): updated recuriting app
</commit_message>
<xml_diff>
--- a/Streamlit Version/Hiring Folder.xlsx
+++ b/Streamlit Version/Hiring Folder.xlsx
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general"/>
@@ -90,6 +95,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,7 +558,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -1160,6 +1166,69 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Contacted 15/06/2026
+Ms yugen, 15/11/1991, turning 35. Last Drawn : 3,800 ( basic ). Reasons for Leaving : the outlet is closing.  2 months notice period, expected salary, anything above 3,800. Open to work on the weekends and public holidays, is perfectly okay with an assistant manager, inorder to progress slowly and learn the ins and out.  wants to have at least 6 off days a month, 5.5 work week. Most number of people managed, 15 under ( 3 kitchen + front of the house ), she wants to manage more people, currently only running with 2 crew and wants more to manage. Bost mos burger and paris baguette had managed mutiple resturants at once due to lack of managers so managed 2 stores stimotaniously, for mos burger have been to all of it, for mos burger they only allow the outlet manager to do ordering and stock take.  have done stock take all the way to audits and checks, P&amp;L meetings, has been throught the whole specturm, from service crew, line cook then resturant manager.</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Contacted</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Yugenthiri_Paramanandan_82616551_Assistant_Restaurant_Manager_Yugenthiri_Paramanandan_Assistant_Restaurant_Manager_Fast_Food_2026-06-15.pdf</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>resumes/Yugenthiri_Paramanandan_82616551_Assistant_Restaurant_Manager_Yugenthiri_Paramanandan_Assistant_Restaurant_Manager_Fast_Food_2026-06-15.pdf</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1171,7 +1240,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -2343,6 +2412,191 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:53:18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>candidate added</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>New candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:53:18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>resume uploaded</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>resumes/Yugenthiri_Paramanandan_82616551_Assistant_Restaurant_Manager_Yugenthiri_Paramanandan_Assistant_Restaurant_Manager_Fast_Food_2026-06-15.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:09:44</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>result changed</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Pending -&gt; Contacted</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:09:44</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>candidate updated</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>CDD details save</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:48:25</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>candidate updated</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Assistant Restaurant Manager</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>assistant_restaurant_manager_82616551</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Yugenthiri Paramanandan</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>82616551</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>CDD details save</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>